<commit_message>
Render mixed-font cells faithfully and apply Jeuz's final workbooks
Cells that mix fonts within their text (e.g. a bold label with an
italic "(2)" footnote) were rendered with the cell's font only, so
italic runs showed as bold. Render each run with its own weight,
style, size, and color, and add a self-check for it. Replace the
four models with Jeuz's final files and update the honors line to
"Honorable Mention, Expected December 2026".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Discounted Cash Flow Analysis.xlsx
+++ b/docs/Discounted Cash Flow Analysis.xlsx
@@ -1026,7 +1026,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="150">
+  <cellXfs count="149">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1155,14 +1155,13 @@
     <xf borderId="1" fillId="3" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="3" fillId="3" fontId="8" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="3" fontId="11" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="3" fillId="3" fontId="8" numFmtId="167" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="3" fillId="3" fontId="8" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="11" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="5" fillId="3" fontId="8" numFmtId="165" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="8" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right"/>
     </xf>
     <xf borderId="6" fillId="3" fontId="11" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="8" fillId="3" fontId="8" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="8" fillId="3" fontId="8" numFmtId="166" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="6" fillId="3" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="8" fillId="3" fontId="6" numFmtId="165" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
@@ -2696,7 +2695,7 @@
         <v>47</v>
       </c>
       <c r="J29" s="10"/>
-      <c r="K29" s="81">
+      <c r="K29" s="61">
         <f>K20</f>
         <v>12816.40599</v>
       </c>
@@ -2714,7 +2713,7 @@
       <c r="A30" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="B30" s="82">
+      <c r="B30" s="81">
         <v>6.6</v>
       </c>
       <c r="C30" s="18"/>
@@ -2725,11 +2724,11 @@
         <v>120.6</v>
       </c>
       <c r="H30" s="18"/>
-      <c r="I30" s="83" t="s">
+      <c r="I30" s="82" t="s">
         <v>40</v>
       </c>
       <c r="J30" s="10"/>
-      <c r="K30" s="84">
+      <c r="K30" s="83">
         <f>((K27*K28)-(K29*(1+K28)^0.5))/(K27+(K29*(1+K28)^0.5))</f>
         <v>0.015923369</v>
       </c>
@@ -2778,15 +2777,15 @@
       <c r="A32" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="B32" s="85">
+      <c r="B32" s="84">
         <f>(1)/(1+K21)^(5)</f>
         <v>0.5810071205</v>
       </c>
       <c r="C32" s="18"/>
-      <c r="D32" s="86" t="s">
+      <c r="D32" s="85" t="s">
         <v>52</v>
       </c>
-      <c r="G32" s="87">
+      <c r="G32" s="86">
         <f>G27-G28-G30+G31</f>
         <v>130845.4133</v>
       </c>
@@ -2810,7 +2809,7 @@
       <c r="A33" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="B33" s="88">
+      <c r="B33" s="87">
         <f>B31*B32</f>
         <v>80848.48704</v>
       </c>
@@ -2825,7 +2824,7 @@
       <c r="I33" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="K33" s="89">
+      <c r="K33" s="88">
         <f>B36</f>
         <v>121756.2133</v>
       </c>
@@ -2843,17 +2842,17 @@
       <c r="A34" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="B34" s="90">
+      <c r="B34" s="89">
         <f>B33/B36</f>
         <v>0.6640193946</v>
       </c>
       <c r="C34" s="18"/>
-      <c r="D34" s="91" t="s">
+      <c r="D34" s="90" t="s">
         <v>57</v>
       </c>
       <c r="E34" s="24"/>
       <c r="F34" s="24"/>
-      <c r="G34" s="92">
+      <c r="G34" s="91">
         <f>G32/G33</f>
         <v>7.281888432</v>
       </c>
@@ -2884,11 +2883,11 @@
       <c r="F35" s="18"/>
       <c r="G35" s="18"/>
       <c r="H35" s="18"/>
-      <c r="I35" s="93" t="s">
+      <c r="I35" s="92" t="s">
         <v>53</v>
       </c>
       <c r="J35" s="10"/>
-      <c r="K35" s="94">
+      <c r="K35" s="93">
         <f>K33/K34</f>
         <v>7.540064856</v>
       </c>
@@ -2903,10 +2902,10 @@
       <c r="T35" s="18"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="91" t="s">
+      <c r="A36" s="90" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="92">
+      <c r="B36" s="91">
         <f>B27+B33</f>
         <v>121756.2133</v>
       </c>
@@ -2930,7 +2929,7 @@
       <c r="T36" s="18"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="95" t="s">
+      <c r="A37" s="94" t="s">
         <v>59</v>
       </c>
       <c r="C37" s="18"/>
@@ -2953,7 +2952,7 @@
       <c r="T37" s="18"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="95" t="s">
+      <c r="A38" s="94" t="s">
         <v>60</v>
       </c>
       <c r="C38" s="18"/>
@@ -2976,7 +2975,7 @@
       <c r="T38" s="18"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="95" t="s">
+      <c r="A39" s="94" t="s">
         <v>61</v>
       </c>
       <c r="C39" s="18"/>
@@ -2999,12 +2998,12 @@
       <c r="T39" s="18"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="95" t="s">
+      <c r="A40" s="94" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="96" t="s">
+      <c r="A41" s="95" t="s">
         <v>63</v>
       </c>
     </row>
@@ -4028,7 +4027,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="96" t="s">
         <v>64</v>
       </c>
       <c r="B1" s="2"/>
@@ -4040,8 +4039,8 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="3"/>
-      <c r="K1" s="98"/>
-      <c r="L1" s="98"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
       <c r="O1" s="4"/>
@@ -4064,8 +4063,8 @@
       <c r="H2" s="10"/>
       <c r="I2" s="10"/>
       <c r="J2" s="11"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="98"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
@@ -4082,7 +4081,7 @@
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="99" t="s">
+      <c r="E3" s="98" t="s">
         <v>5</v>
       </c>
       <c r="F3" s="14" t="s">
@@ -4092,8 +4091,8 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="98"/>
-      <c r="L3" s="98"/>
+      <c r="K3" s="97"/>
+      <c r="L3" s="97"/>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
@@ -4113,7 +4112,7 @@
       <c r="D4" s="20">
         <v>2025.0</v>
       </c>
-      <c r="E4" s="100">
+      <c r="E4" s="99">
         <v>2026.0</v>
       </c>
       <c r="F4" s="20">
@@ -4128,11 +4127,11 @@
       <c r="I4" s="20">
         <v>2030.0</v>
       </c>
-      <c r="J4" s="101">
+      <c r="J4" s="100">
         <v>2031.0</v>
       </c>
-      <c r="K4" s="98"/>
-      <c r="L4" s="98"/>
+      <c r="K4" s="97"/>
+      <c r="L4" s="97"/>
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
       <c r="O4" s="18"/>
@@ -4145,35 +4144,35 @@
       <c r="A5" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="102">
+      <c r="B5" s="101">
         <v>80169.5</v>
       </c>
-      <c r="C5" s="102">
+      <c r="C5" s="101">
         <v>83120.1</v>
       </c>
-      <c r="D5" s="102">
+      <c r="D5" s="101">
         <v>86483.0</v>
       </c>
-      <c r="E5" s="103">
+      <c r="E5" s="102">
         <v>90755.0</v>
       </c>
-      <c r="F5" s="102">
+      <c r="F5" s="101">
         <v>95707.0</v>
       </c>
-      <c r="G5" s="102">
+      <c r="G5" s="101">
         <v>100088.0</v>
       </c>
-      <c r="H5" s="102">
+      <c r="H5" s="101">
         <v>104091.52</v>
       </c>
-      <c r="I5" s="102">
+      <c r="I5" s="101">
         <v>107734.72</v>
       </c>
-      <c r="J5" s="89">
+      <c r="J5" s="88">
         <v>110966.76</v>
       </c>
-      <c r="K5" s="98"/>
-      <c r="L5" s="98"/>
+      <c r="K5" s="97"/>
+      <c r="L5" s="97"/>
       <c r="M5" s="18"/>
       <c r="N5" s="18"/>
       <c r="O5" s="18"/>
@@ -4187,36 +4186,36 @@
       <c r="A6" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="104">
+      <c r="B6" s="103">
         <v>52669.7</v>
       </c>
-      <c r="C6" s="104">
+      <c r="C6" s="103">
         <v>51742.5</v>
       </c>
-      <c r="D6" s="104">
+      <c r="D6" s="103">
         <v>54837.9</v>
       </c>
-      <c r="E6" s="105">
+      <c r="E6" s="104">
         <f t="shared" ref="E6:J6" si="1">E5*E7</f>
         <v>57546.72727</v>
       </c>
-      <c r="F6" s="104">
+      <c r="F6" s="103">
         <f t="shared" si="1"/>
         <v>60686.73491</v>
       </c>
-      <c r="G6" s="104">
+      <c r="G6" s="103">
         <f t="shared" si="1"/>
         <v>63464.67786</v>
       </c>
-      <c r="H6" s="104">
+      <c r="H6" s="103">
         <f t="shared" si="1"/>
         <v>66003.26497</v>
       </c>
-      <c r="I6" s="104">
+      <c r="I6" s="103">
         <f t="shared" si="1"/>
         <v>68313.37722</v>
       </c>
-      <c r="J6" s="106">
+      <c r="J6" s="105">
         <f t="shared" si="1"/>
         <v>70362.77752</v>
       </c>
@@ -4233,39 +4232,39 @@
       <c r="A7" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="107">
+      <c r="B7" s="106">
         <f t="shared" ref="B7:D7" si="2">B6/B5</f>
         <v>0.6569792752</v>
       </c>
-      <c r="C7" s="107">
+      <c r="C7" s="106">
         <f t="shared" si="2"/>
         <v>0.6225028603</v>
       </c>
-      <c r="D7" s="107">
+      <c r="D7" s="106">
         <f t="shared" si="2"/>
         <v>0.6340887805</v>
       </c>
-      <c r="E7" s="108">
+      <c r="E7" s="107">
         <f t="shared" ref="E7:J7" si="3">D7</f>
         <v>0.6340887805</v>
       </c>
-      <c r="F7" s="107">
+      <c r="F7" s="106">
         <f t="shared" si="3"/>
         <v>0.6340887805</v>
       </c>
-      <c r="G7" s="107">
+      <c r="G7" s="106">
         <f t="shared" si="3"/>
         <v>0.6340887805</v>
       </c>
-      <c r="H7" s="107">
+      <c r="H7" s="106">
         <f t="shared" si="3"/>
         <v>0.6340887805</v>
       </c>
-      <c r="I7" s="107">
+      <c r="I7" s="106">
         <f t="shared" si="3"/>
         <v>0.6340887805</v>
       </c>
-      <c r="J7" s="109">
+      <c r="J7" s="108">
         <f t="shared" si="3"/>
         <v>0.6340887805</v>
       </c>
@@ -4280,14 +4279,14 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="31"/>
-      <c r="B8" s="110"/>
-      <c r="C8" s="110"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
-      <c r="F8" s="110"/>
-      <c r="G8" s="110"/>
-      <c r="H8" s="110"/>
-      <c r="I8" s="110"/>
+      <c r="B8" s="109"/>
+      <c r="C8" s="109"/>
+      <c r="D8" s="109"/>
+      <c r="E8" s="110"/>
+      <c r="F8" s="109"/>
+      <c r="G8" s="109"/>
+      <c r="H8" s="109"/>
+      <c r="I8" s="109"/>
       <c r="J8" s="77"/>
       <c r="M8" s="18"/>
       <c r="N8" s="18"/>
@@ -4305,7 +4304,7 @@
       <c r="B9" s="35"/>
       <c r="C9" s="35"/>
       <c r="D9" s="35"/>
-      <c r="E9" s="112"/>
+      <c r="E9" s="111"/>
       <c r="F9" s="35"/>
       <c r="G9" s="35"/>
       <c r="H9" s="35"/>
@@ -4335,7 +4334,7 @@
       <c r="D10" s="42">
         <v>8400.98</v>
       </c>
-      <c r="E10" s="113">
+      <c r="E10" s="112">
         <f t="shared" ref="E10:J10" si="4">(E5/365)*E27</f>
         <v>8815.963136</v>
       </c>
@@ -4383,7 +4382,7 @@
       <c r="D11" s="42">
         <v>8971.75</v>
       </c>
-      <c r="E11" s="113">
+      <c r="E11" s="112">
         <f t="shared" ref="E11:J11" si="5">(E6/365)*E28</f>
         <v>9414.927457</v>
       </c>
@@ -4431,7 +4430,7 @@
       <c r="D12" s="60">
         <v>1756.24</v>
       </c>
-      <c r="E12" s="114">
+      <c r="E12" s="113">
         <f t="shared" ref="E12:J12" si="6">E5*E29</f>
         <v>1842.992972</v>
       </c>
@@ -4482,7 +4481,7 @@
         <f t="shared" si="7"/>
         <v>19128.97</v>
       </c>
-      <c r="E13" s="115">
+      <c r="E13" s="114">
         <f t="shared" si="7"/>
         <v>20073.88356</v>
       </c>
@@ -4502,7 +4501,7 @@
         <f t="shared" si="7"/>
         <v>23829.58763</v>
       </c>
-      <c r="J13" s="88">
+      <c r="J13" s="87">
         <f t="shared" si="7"/>
         <v>24544.4749</v>
       </c>
@@ -4522,7 +4521,7 @@
       <c r="B14" s="35"/>
       <c r="C14" s="35"/>
       <c r="D14" s="35"/>
-      <c r="E14" s="112"/>
+      <c r="E14" s="111"/>
       <c r="F14" s="35"/>
       <c r="G14" s="35"/>
       <c r="H14" s="35"/>
@@ -4546,7 +4545,7 @@
       <c r="B15" s="35"/>
       <c r="C15" s="35"/>
       <c r="D15" s="35"/>
-      <c r="E15" s="112"/>
+      <c r="E15" s="111"/>
       <c r="F15" s="35"/>
       <c r="G15" s="35"/>
       <c r="H15" s="35"/>
@@ -4576,7 +4575,7 @@
       <c r="D16" s="42">
         <v>6143.84</v>
       </c>
-      <c r="E16" s="113">
+      <c r="E16" s="112">
         <f t="shared" ref="E16:J16" si="8">(E6/365)*E32</f>
         <v>6447.327211</v>
       </c>
@@ -4623,7 +4622,7 @@
       <c r="D17" s="42">
         <v>2418.84</v>
       </c>
-      <c r="E17" s="113">
+      <c r="E17" s="112">
         <f t="shared" ref="E17:J17" si="9">E5*E33</f>
         <v>2538.323418</v>
       </c>
@@ -4670,7 +4669,7 @@
       <c r="D18" s="60">
         <v>3878.7</v>
       </c>
-      <c r="E18" s="114">
+      <c r="E18" s="113">
         <f t="shared" ref="E18:J18" si="10">E5*E34</f>
         <v>4070.29611</v>
       </c>
@@ -4720,7 +4719,7 @@
         <f t="shared" si="11"/>
         <v>12441.38</v>
       </c>
-      <c r="E19" s="115">
+      <c r="E19" s="114">
         <f t="shared" si="11"/>
         <v>13055.94674</v>
       </c>
@@ -4740,7 +4739,7 @@
         <f t="shared" si="11"/>
         <v>15498.63662</v>
       </c>
-      <c r="J19" s="88">
+      <c r="J19" s="87">
         <f t="shared" si="11"/>
         <v>15963.59549</v>
       </c>
@@ -4759,7 +4758,7 @@
       <c r="B20" s="35"/>
       <c r="C20" s="35"/>
       <c r="D20" s="35"/>
-      <c r="E20" s="112"/>
+      <c r="E20" s="111"/>
       <c r="F20" s="35"/>
       <c r="G20" s="35"/>
       <c r="H20" s="35"/>
@@ -4791,7 +4790,7 @@
         <f t="shared" si="12"/>
         <v>6687.59</v>
       </c>
-      <c r="E21" s="115">
+      <c r="E21" s="114">
         <f t="shared" si="12"/>
         <v>7017.936825</v>
       </c>
@@ -4811,7 +4810,7 @@
         <f t="shared" si="12"/>
         <v>8330.951009</v>
       </c>
-      <c r="J21" s="88">
+      <c r="J21" s="87">
         <f t="shared" si="12"/>
         <v>8580.879416</v>
       </c>
@@ -4841,7 +4840,7 @@
         <f t="shared" si="13"/>
         <v>0.07732837668</v>
       </c>
-      <c r="E22" s="116">
+      <c r="E22" s="115">
         <f t="shared" si="13"/>
         <v>0.07732837668</v>
       </c>
@@ -4861,7 +4860,7 @@
         <f t="shared" si="13"/>
         <v>0.07732837668</v>
       </c>
-      <c r="J22" s="90">
+      <c r="J22" s="89">
         <f t="shared" si="13"/>
         <v>0.07732837668</v>
       </c>
@@ -4888,7 +4887,7 @@
         <f t="shared" si="14"/>
         <v>1281.25</v>
       </c>
-      <c r="E23" s="117">
+      <c r="E23" s="116">
         <f t="shared" si="14"/>
         <v>330.3468252</v>
       </c>
@@ -4908,7 +4907,7 @@
         <f t="shared" si="14"/>
         <v>281.7227419</v>
       </c>
-      <c r="J23" s="118">
+      <c r="J23" s="117">
         <f t="shared" si="14"/>
         <v>249.9284065</v>
       </c>
@@ -4924,14 +4923,14 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="31"/>
-      <c r="B24" s="110"/>
-      <c r="C24" s="110"/>
-      <c r="D24" s="110"/>
-      <c r="E24" s="111"/>
-      <c r="F24" s="110"/>
-      <c r="G24" s="110"/>
-      <c r="H24" s="110"/>
-      <c r="I24" s="110"/>
+      <c r="B24" s="109"/>
+      <c r="C24" s="109"/>
+      <c r="D24" s="109"/>
+      <c r="E24" s="110"/>
+      <c r="F24" s="109"/>
+      <c r="G24" s="109"/>
+      <c r="H24" s="109"/>
+      <c r="I24" s="109"/>
       <c r="J24" s="77"/>
       <c r="K24" s="18"/>
       <c r="L24" s="18"/>
@@ -4944,13 +4943,13 @@
       <c r="S24" s="18"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="119" t="s">
+      <c r="A25" s="118" t="s">
         <v>80</v>
       </c>
       <c r="B25" s="35"/>
       <c r="C25" s="35"/>
       <c r="D25" s="35"/>
-      <c r="E25" s="112"/>
+      <c r="E25" s="111"/>
       <c r="F25" s="35"/>
       <c r="G25" s="35"/>
       <c r="H25" s="35"/>
@@ -4973,7 +4972,7 @@
       <c r="B26" s="35"/>
       <c r="C26" s="35"/>
       <c r="D26" s="35"/>
-      <c r="E26" s="112"/>
+      <c r="E26" s="111"/>
       <c r="F26" s="35"/>
       <c r="G26" s="35"/>
       <c r="H26" s="35"/>
@@ -5005,7 +5004,7 @@
         <f t="shared" si="15"/>
         <v>35.45619023</v>
       </c>
-      <c r="E27" s="113">
+      <c r="E27" s="112">
         <f t="shared" ref="E27:J27" si="16">D27</f>
         <v>35.45619023</v>
       </c>
@@ -5055,7 +5054,7 @@
         <f t="shared" si="17"/>
         <v>59.71579419</v>
       </c>
-      <c r="E28" s="113">
+      <c r="E28" s="112">
         <f t="shared" ref="E28:J28" si="18">D28</f>
         <v>59.71579419</v>
       </c>
@@ -5093,35 +5092,35 @@
       <c r="A29" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="B29" s="120">
+      <c r="B29" s="119">
         <f t="shared" ref="B29:D29" si="19">B12/B5</f>
         <v>0.0137168125</v>
       </c>
-      <c r="C29" s="120">
+      <c r="C29" s="119">
         <f t="shared" si="19"/>
         <v>0.01595462469</v>
       </c>
-      <c r="D29" s="120">
+      <c r="D29" s="119">
         <f t="shared" si="19"/>
         <v>0.02030734364</v>
       </c>
-      <c r="E29" s="121">
+      <c r="E29" s="120">
         <f t="shared" ref="E29:J29" si="20">D29</f>
         <v>0.02030734364</v>
       </c>
-      <c r="F29" s="120">
+      <c r="F29" s="119">
         <f t="shared" si="20"/>
         <v>0.02030734364</v>
       </c>
-      <c r="G29" s="120">
+      <c r="G29" s="119">
         <f t="shared" si="20"/>
         <v>0.02030734364</v>
       </c>
-      <c r="H29" s="120">
+      <c r="H29" s="119">
         <f t="shared" si="20"/>
         <v>0.02030734364</v>
       </c>
-      <c r="I29" s="120">
+      <c r="I29" s="119">
         <f t="shared" si="20"/>
         <v>0.02030734364</v>
       </c>
@@ -5144,7 +5143,7 @@
       <c r="B30" s="35"/>
       <c r="C30" s="35"/>
       <c r="D30" s="35"/>
-      <c r="E30" s="112"/>
+      <c r="E30" s="111"/>
       <c r="F30" s="35"/>
       <c r="G30" s="35"/>
       <c r="H30" s="35"/>
@@ -5167,7 +5166,7 @@
       <c r="B31" s="35"/>
       <c r="C31" s="35"/>
       <c r="D31" s="35"/>
-      <c r="E31" s="112"/>
+      <c r="E31" s="111"/>
       <c r="F31" s="35"/>
       <c r="G31" s="35"/>
       <c r="H31" s="35"/>
@@ -5199,7 +5198,7 @@
         <f t="shared" si="21"/>
         <v>40.89328001</v>
       </c>
-      <c r="E32" s="113">
+      <c r="E32" s="112">
         <f t="shared" ref="E32:J32" si="22">D32</f>
         <v>40.89328001</v>
       </c>
@@ -5237,35 +5236,35 @@
       <c r="A33" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B33" s="120">
+      <c r="B33" s="119">
         <f t="shared" ref="B33:D33" si="23">B17/B5</f>
         <v>0.01919707619</v>
       </c>
-      <c r="C33" s="120">
+      <c r="C33" s="119">
         <f t="shared" si="23"/>
         <v>0.02498902191</v>
       </c>
-      <c r="D33" s="120">
+      <c r="D33" s="119">
         <f t="shared" si="23"/>
         <v>0.027968965</v>
       </c>
-      <c r="E33" s="121">
+      <c r="E33" s="120">
         <f t="shared" ref="E33:J33" si="24">D33</f>
         <v>0.027968965</v>
       </c>
-      <c r="F33" s="120">
+      <c r="F33" s="119">
         <f t="shared" si="24"/>
         <v>0.027968965</v>
       </c>
-      <c r="G33" s="120">
+      <c r="G33" s="119">
         <f t="shared" si="24"/>
         <v>0.027968965</v>
       </c>
-      <c r="H33" s="120">
+      <c r="H33" s="119">
         <f t="shared" si="24"/>
         <v>0.027968965</v>
       </c>
-      <c r="I33" s="120">
+      <c r="I33" s="119">
         <f t="shared" si="24"/>
         <v>0.027968965</v>
       </c>
@@ -5287,39 +5286,39 @@
       <c r="A34" s="52" t="s">
         <v>86</v>
       </c>
-      <c r="B34" s="122">
+      <c r="B34" s="121">
         <f t="shared" ref="B34:D34" si="25">B18/B5</f>
         <v>0.06466524052</v>
       </c>
-      <c r="C34" s="122">
+      <c r="C34" s="121">
         <f t="shared" si="25"/>
         <v>0.05008836611</v>
       </c>
-      <c r="D34" s="122">
+      <c r="D34" s="121">
         <f t="shared" si="25"/>
         <v>0.04484927674</v>
       </c>
-      <c r="E34" s="123">
+      <c r="E34" s="122">
         <f t="shared" ref="E34:J34" si="26">D34</f>
         <v>0.04484927674</v>
       </c>
-      <c r="F34" s="122">
+      <c r="F34" s="121">
         <f t="shared" si="26"/>
         <v>0.04484927674</v>
       </c>
-      <c r="G34" s="122">
+      <c r="G34" s="121">
         <f t="shared" si="26"/>
         <v>0.04484927674</v>
       </c>
-      <c r="H34" s="122">
+      <c r="H34" s="121">
         <f t="shared" si="26"/>
         <v>0.04484927674</v>
       </c>
-      <c r="I34" s="122">
+      <c r="I34" s="121">
         <f t="shared" si="26"/>
         <v>0.04484927674</v>
       </c>
-      <c r="J34" s="124">
+      <c r="J34" s="123">
         <f t="shared" si="26"/>
         <v>0.04484927674</v>
       </c>
@@ -5355,16 +5354,16 @@
       <c r="S35" s="18"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="125" t="s">
+      <c r="A36" s="124" t="s">
         <v>87</v>
       </c>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="3"/>
-      <c r="E36" s="126"/>
-      <c r="F36" s="126"/>
-      <c r="G36" s="126"/>
-      <c r="H36" s="126"/>
+      <c r="E36" s="125"/>
+      <c r="F36" s="125"/>
+      <c r="G36" s="125"/>
+      <c r="H36" s="125"/>
       <c r="I36" s="18"/>
       <c r="J36" s="18"/>
       <c r="K36" s="18"/>
@@ -5385,9 +5384,9 @@
       <c r="C37" s="10"/>
       <c r="D37" s="11"/>
       <c r="E37" s="12"/>
-      <c r="F37" s="126"/>
-      <c r="G37" s="126"/>
-      <c r="H37" s="126"/>
+      <c r="F37" s="125"/>
+      <c r="G37" s="125"/>
+      <c r="H37" s="125"/>
       <c r="I37" s="18"/>
       <c r="J37" s="18"/>
       <c r="K37" s="18"/>
@@ -5402,19 +5401,19 @@
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="73"/>
-      <c r="B38" s="127" t="s">
+      <c r="B38" s="126" t="s">
         <v>89</v>
       </c>
-      <c r="C38" s="128" t="s">
+      <c r="C38" s="127" t="s">
         <v>90</v>
       </c>
-      <c r="D38" s="129" t="s">
+      <c r="D38" s="128" t="s">
         <v>91</v>
       </c>
-      <c r="E38" s="98"/>
-      <c r="F38" s="126"/>
-      <c r="G38" s="126"/>
-      <c r="H38" s="126"/>
+      <c r="E38" s="97"/>
+      <c r="F38" s="125"/>
+      <c r="G38" s="125"/>
+      <c r="H38" s="125"/>
       <c r="I38" s="18"/>
       <c r="J38" s="18"/>
       <c r="K38" s="18"/>
@@ -5431,19 +5430,19 @@
       <c r="A39" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="B39" s="102">
+      <c r="B39" s="101">
         <v>2557.3</v>
       </c>
-      <c r="C39" s="102">
+      <c r="C39" s="101">
         <v>173.9</v>
       </c>
       <c r="D39" s="78">
         <v>0.068</v>
       </c>
-      <c r="E39" s="130"/>
-      <c r="F39" s="126"/>
-      <c r="G39" s="126"/>
-      <c r="H39" s="126"/>
+      <c r="E39" s="129"/>
+      <c r="F39" s="125"/>
+      <c r="G39" s="125"/>
+      <c r="H39" s="125"/>
       <c r="I39" s="18"/>
       <c r="J39" s="18"/>
       <c r="K39" s="18"/>
@@ -5460,301 +5459,301 @@
       <c r="A40" s="31" t="s">
         <v>93</v>
       </c>
-      <c r="B40" s="104">
+      <c r="B40" s="103">
         <v>1638.4</v>
       </c>
-      <c r="C40" s="104">
+      <c r="C40" s="103">
         <v>146.3</v>
       </c>
-      <c r="D40" s="131">
+      <c r="D40" s="130">
         <v>0.0893</v>
       </c>
-      <c r="E40" s="130"/>
-      <c r="F40" s="126"/>
-      <c r="G40" s="126"/>
-      <c r="H40" s="126"/>
+      <c r="E40" s="129"/>
+      <c r="F40" s="125"/>
+      <c r="G40" s="125"/>
+      <c r="H40" s="125"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="80" t="s">
         <v>94</v>
       </c>
-      <c r="B41" s="132">
+      <c r="B41" s="131">
         <v>1040.0</v>
       </c>
-      <c r="C41" s="132">
+      <c r="C41" s="131">
         <v>62.0</v>
       </c>
-      <c r="D41" s="133">
+      <c r="D41" s="132">
         <v>0.0596</v>
       </c>
-      <c r="E41" s="130"/>
-      <c r="F41" s="126"/>
-      <c r="G41" s="126"/>
-      <c r="H41" s="126"/>
-      <c r="I41" s="96"/>
+      <c r="E41" s="129"/>
+      <c r="F41" s="125"/>
+      <c r="G41" s="125"/>
+      <c r="H41" s="125"/>
+      <c r="I41" s="95"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="80" t="s">
         <v>95</v>
       </c>
-      <c r="B42" s="134">
+      <c r="B42" s="133">
         <f>SUM(B39:B41)</f>
         <v>5235.7</v>
       </c>
-      <c r="C42" s="135"/>
-      <c r="D42" s="136"/>
-      <c r="F42" s="126"/>
-      <c r="G42" s="126"/>
-      <c r="H42" s="126"/>
-      <c r="I42" s="96"/>
+      <c r="C42" s="134"/>
+      <c r="D42" s="135"/>
+      <c r="F42" s="125"/>
+      <c r="G42" s="125"/>
+      <c r="H42" s="125"/>
+      <c r="I42" s="95"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="137"/>
-      <c r="B43" s="110"/>
-      <c r="C43" s="110"/>
+      <c r="A43" s="136"/>
+      <c r="B43" s="109"/>
+      <c r="C43" s="109"/>
       <c r="D43" s="77"/>
-      <c r="F43" s="126"/>
-      <c r="G43" s="126"/>
-      <c r="H43" s="126"/>
+      <c r="F43" s="125"/>
+      <c r="G43" s="125"/>
+      <c r="H43" s="125"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="80" t="s">
         <v>96</v>
       </c>
-      <c r="B44" s="138">
+      <c r="B44" s="137">
         <f>((B39/B42)*D39)+((B40/B42)*D40)+((B41/B42)*D41)</f>
         <v>0.07299683328</v>
       </c>
-      <c r="C44" s="110"/>
+      <c r="C44" s="109"/>
       <c r="D44" s="77"/>
-      <c r="F44" s="126"/>
-      <c r="G44" s="126"/>
-      <c r="H44" s="126"/>
+      <c r="F44" s="125"/>
+      <c r="G44" s="125"/>
+      <c r="H44" s="125"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="80" t="s">
         <v>97</v>
       </c>
-      <c r="B45" s="139">
+      <c r="B45" s="138">
         <f>B44*(1-0.25)</f>
         <v>0.05474762496</v>
       </c>
-      <c r="C45" s="135"/>
-      <c r="D45" s="136"/>
-      <c r="F45" s="126"/>
-      <c r="G45" s="126"/>
-      <c r="H45" s="126"/>
+      <c r="C45" s="134"/>
+      <c r="D45" s="135"/>
+      <c r="F45" s="125"/>
+      <c r="G45" s="125"/>
+      <c r="H45" s="125"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="F46" s="126"/>
-      <c r="G46" s="126"/>
-      <c r="H46" s="126"/>
+      <c r="F46" s="125"/>
+      <c r="G46" s="125"/>
+      <c r="H46" s="125"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="125" t="s">
+      <c r="A47" s="124" t="s">
         <v>98</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="3"/>
-      <c r="F47" s="126"/>
-      <c r="G47" s="126"/>
-      <c r="H47" s="126"/>
+      <c r="F47" s="125"/>
+      <c r="G47" s="125"/>
+      <c r="H47" s="125"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="140" t="s">
+      <c r="A48" s="139" t="s">
         <v>99</v>
       </c>
-      <c r="B48" s="141" t="s">
+      <c r="B48" s="140" t="s">
         <v>100</v>
       </c>
-      <c r="C48" s="141" t="s">
+      <c r="C48" s="140" t="s">
         <v>101</v>
       </c>
-      <c r="D48" s="129" t="s">
+      <c r="D48" s="128" t="s">
         <v>102</v>
       </c>
-      <c r="F48" s="126"/>
-      <c r="G48" s="126"/>
-      <c r="H48" s="126"/>
+      <c r="F48" s="125"/>
+      <c r="G48" s="125"/>
+      <c r="H48" s="125"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="31" t="s">
         <v>103</v>
       </c>
-      <c r="B49" s="110">
+      <c r="B49" s="109">
         <v>0.82</v>
       </c>
-      <c r="C49" s="142">
+      <c r="C49" s="141">
         <v>0.1997</v>
       </c>
-      <c r="D49" s="143">
+      <c r="D49" s="142">
         <f t="shared" ref="D49:D51" si="27">(B49)/(1+C49*(1-0.25))</f>
         <v>0.7131830141</v>
       </c>
-      <c r="F49" s="126"/>
-      <c r="G49" s="126"/>
-      <c r="H49" s="126"/>
+      <c r="F49" s="125"/>
+      <c r="G49" s="125"/>
+      <c r="H49" s="125"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="B50" s="110">
+      <c r="B50" s="109">
         <v>0.74</v>
       </c>
-      <c r="C50" s="142">
+      <c r="C50" s="141">
         <v>0.1266</v>
       </c>
-      <c r="D50" s="143">
+      <c r="D50" s="142">
         <f t="shared" si="27"/>
         <v>0.6758299466</v>
       </c>
-      <c r="F50" s="126"/>
-      <c r="G50" s="126"/>
-      <c r="H50" s="126"/>
+      <c r="F50" s="125"/>
+      <c r="G50" s="125"/>
+      <c r="H50" s="125"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="31" t="s">
         <v>105</v>
       </c>
-      <c r="B51" s="110">
+      <c r="B51" s="109">
         <v>0.38</v>
       </c>
-      <c r="C51" s="142">
+      <c r="C51" s="141">
         <v>0.3421</v>
       </c>
-      <c r="D51" s="143">
+      <c r="D51" s="142">
         <f t="shared" si="27"/>
         <v>0.3024093269</v>
       </c>
-      <c r="F51" s="126"/>
-      <c r="G51" s="126"/>
-      <c r="H51" s="126"/>
+      <c r="F51" s="125"/>
+      <c r="G51" s="125"/>
+      <c r="H51" s="125"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="31"/>
-      <c r="B52" s="110"/>
-      <c r="C52" s="110"/>
+      <c r="B52" s="109"/>
+      <c r="C52" s="109"/>
       <c r="D52" s="77"/>
-      <c r="F52" s="126"/>
-      <c r="G52" s="126"/>
-      <c r="H52" s="126"/>
+      <c r="F52" s="125"/>
+      <c r="G52" s="125"/>
+      <c r="H52" s="125"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="80" t="s">
         <v>106</v>
       </c>
-      <c r="B53" s="144">
+      <c r="B53" s="143">
         <f>D50</f>
         <v>0.6758299466</v>
       </c>
-      <c r="C53" s="110"/>
+      <c r="C53" s="109"/>
       <c r="D53" s="77"/>
-      <c r="F53" s="126"/>
-      <c r="G53" s="126"/>
-      <c r="H53" s="126"/>
+      <c r="F53" s="125"/>
+      <c r="G53" s="125"/>
+      <c r="H53" s="125"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="31" t="s">
         <v>107</v>
       </c>
-      <c r="B54" s="145">
+      <c r="B54" s="144">
         <f>B53*(1+C49*(1-0.25))</f>
         <v>0.7770523768</v>
       </c>
-      <c r="C54" s="110"/>
+      <c r="C54" s="109"/>
       <c r="D54" s="77"/>
-      <c r="F54" s="126"/>
-      <c r="G54" s="126"/>
-      <c r="H54" s="126"/>
+      <c r="F54" s="125"/>
+      <c r="G54" s="125"/>
+      <c r="H54" s="125"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="31"/>
-      <c r="B55" s="110"/>
-      <c r="C55" s="110"/>
+      <c r="B55" s="109"/>
+      <c r="C55" s="109"/>
       <c r="D55" s="77"/>
-      <c r="F55" s="126"/>
-      <c r="G55" s="126"/>
-      <c r="H55" s="126"/>
+      <c r="F55" s="125"/>
+      <c r="G55" s="125"/>
+      <c r="H55" s="125"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="31" t="s">
         <v>108</v>
       </c>
-      <c r="B56" s="142">
+      <c r="B56" s="141">
         <v>0.0723</v>
       </c>
-      <c r="C56" s="110"/>
+      <c r="C56" s="109"/>
       <c r="D56" s="77"/>
-      <c r="F56" s="126"/>
-      <c r="G56" s="126"/>
-      <c r="H56" s="126"/>
+      <c r="F56" s="125"/>
+      <c r="G56" s="125"/>
+      <c r="H56" s="125"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="31" t="s">
         <v>109</v>
       </c>
-      <c r="B57" s="142">
+      <c r="B57" s="141">
         <v>0.07</v>
       </c>
-      <c r="C57" s="110"/>
+      <c r="C57" s="109"/>
       <c r="D57" s="77"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="80" t="s">
         <v>110</v>
       </c>
-      <c r="B58" s="138">
+      <c r="B58" s="137">
         <v>0.0</v>
       </c>
-      <c r="C58" s="110"/>
+      <c r="C58" s="109"/>
       <c r="D58" s="77"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="146" t="s">
+      <c r="A59" s="145" t="s">
         <v>111</v>
       </c>
-      <c r="B59" s="139">
+      <c r="B59" s="138">
         <f>B56+(B54*B57)+B58</f>
         <v>0.1266936664</v>
       </c>
-      <c r="C59" s="135"/>
-      <c r="D59" s="136"/>
+      <c r="C59" s="134"/>
+      <c r="D59" s="135"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="96" t="s">
+      <c r="A60" s="95" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="96" t="s">
+      <c r="A61" s="95" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="96" t="s">
+      <c r="A62" s="95" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="96" t="s">
+      <c r="A63" s="95" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="96" t="s">
+      <c r="A64" s="95" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="96" t="s">
+      <c r="A65" s="95" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1"/>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="147" t="s">
+      <c r="A67" s="146" t="s">
         <v>118</v>
       </c>
       <c r="B67" s="25"/>
@@ -5763,13 +5762,13 @@
       <c r="A68" s="75" t="s">
         <v>119</v>
       </c>
-      <c r="B68" s="148"/>
+      <c r="B68" s="147"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="B69" s="131">
+      <c r="B69" s="130">
         <v>0.1665</v>
       </c>
     </row>
@@ -5777,7 +5776,7 @@
       <c r="A70" s="31" t="s">
         <v>121</v>
       </c>
-      <c r="B70" s="131">
+      <c r="B70" s="130">
         <v>0.8335</v>
       </c>
     </row>
@@ -5789,7 +5788,7 @@
       <c r="A72" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="B72" s="131">
+      <c r="B72" s="130">
         <f>B45</f>
         <v>0.05474762496</v>
       </c>
@@ -5798,46 +5797,46 @@
       <c r="A73" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="B73" s="131">
+      <c r="B73" s="130">
         <f>B59</f>
         <v>0.1266936664</v>
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="80"/>
-      <c r="B74" s="136"/>
+      <c r="B74" s="135"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="146" t="s">
+      <c r="A75" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="B75" s="149">
+      <c r="B75" s="148">
         <f>(B70*B73)+(B69*B72)</f>
         <v>0.1147146505</v>
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="96" t="s">
+      <c r="A76" s="95" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="96" t="s">
+      <c r="A77" s="95" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="96" t="s">
+      <c r="A78" s="95" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="96" t="s">
+      <c r="A79" s="95" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="96" t="s">
+      <c r="A80" s="95" t="s">
         <v>127</v>
       </c>
     </row>

</xml_diff>